<commit_message>
fix(fsm): correct vision vs ultrasonic responsibilities
- Vision camera is solely responsible for detecting road traffic stuck on the bridge deck.
- Ultrasonic sensors are solely responsible for detecting approaching marine vessels.
- fsm_guard_can_clear_road now only triggers on ultrasonic (or manual operator).
- fsm_guard_road_clear now explicitly requires !vision.vehicle_present before the motor can engage.
</commit_message>
<xml_diff>
--- a/bom/VLB_Group7_BOM.xlsx
+++ b/bom/VLB_Group7_BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ECE_4.2\Microprocessors II\Course project\vertical-lift-bridge\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF2AFCC-6EF7-4571-8146-CB0E29934565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C128A4F-FBD3-44C2-8E8E-32C0FE88303B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43140" yWindow="1830" windowWidth="19200" windowHeight="11715" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -258,12 +258,6 @@
     <t>Main controller</t>
   </si>
   <si>
-    <t>BTS7960 43A H-bridge driver module</t>
-  </si>
-  <si>
-    <t>BTS7960B</t>
-  </si>
-  <si>
     <t>Motor driver — overspec'd for safety margin</t>
   </si>
   <si>
@@ -616,6 +610,12 @@
   </si>
   <si>
     <t>Lead unit: BLUE = manually entered input; BLACK = formula. Adjust E:F cells to scale procurement.</t>
+  </si>
+  <si>
+    <t>L293D H-bridge driver module</t>
+  </si>
+  <si>
+    <t>Motor Driver</t>
   </si>
 </sst>
 </file>
@@ -757,10 +757,6 @@
   </cellStyleXfs>
   <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -785,6 +781,10 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1085,1695 +1085,1695 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
     </row>
     <row r="3" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A3" s="4">
-        <v>1</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="4">
         <v>1450</v>
       </c>
-      <c r="F3" s="7">
-        <v>1</v>
-      </c>
-      <c r="G3" s="8">
+      <c r="F3" s="5">
+        <v>1</v>
+      </c>
+      <c r="G3" s="6">
         <f t="shared" ref="G3:G20" si="0">E3*F3</f>
         <v>1450</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="4">
+      <c r="A4" s="2">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="4">
         <v>600</v>
       </c>
-      <c r="F4" s="7">
-        <v>1</v>
-      </c>
-      <c r="G4" s="8">
+      <c r="F4" s="5">
+        <v>1</v>
+      </c>
+      <c r="G4" s="6">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
+      <c r="A5" s="2">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="4">
         <v>350</v>
       </c>
-      <c r="F5" s="7">
-        <v>1</v>
-      </c>
-      <c r="G5" s="8">
+      <c r="F5" s="5">
+        <v>1</v>
+      </c>
+      <c r="G5" s="6">
         <f t="shared" si="0"/>
         <v>350</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="4">
+      <c r="A6" s="2">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="4">
         <v>0</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="5">
         <v>4</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="4">
+      <c r="A7" s="2">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="4">
         <v>50</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="5">
         <v>8</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="6">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="4">
+      <c r="A8" s="2">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="4">
         <v>80</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="5">
         <v>4</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="6">
         <f t="shared" si="0"/>
         <v>320</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="4">
+      <c r="A9" s="2">
         <v>7</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="4">
         <v>1250</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="5">
         <v>2</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="6">
         <f t="shared" si="0"/>
         <v>2500</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="4">
+      <c r="A10" s="2">
         <v>8</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="4">
         <v>250</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="5">
         <v>2</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="6">
         <f t="shared" si="0"/>
         <v>500</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="4">
+      <c r="A11" s="2">
         <v>9</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="4">
         <v>180</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="5">
         <v>4</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="6">
         <f t="shared" si="0"/>
         <v>720</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="3" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="4">
+      <c r="A12" s="2">
         <v>10</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="4">
         <v>1500</v>
       </c>
-      <c r="F12" s="7">
-        <v>1</v>
-      </c>
-      <c r="G12" s="8">
+      <c r="F12" s="5">
+        <v>1</v>
+      </c>
+      <c r="G12" s="6">
         <f t="shared" si="0"/>
         <v>1500</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="H12" s="3" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" s="4">
+      <c r="A13" s="2">
         <v>11</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="4">
         <v>80</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="5">
         <v>4</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="6">
         <f t="shared" si="0"/>
         <v>320</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="3" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" s="4">
+      <c r="A14" s="2">
         <v>12</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="4">
         <v>1400</v>
       </c>
-      <c r="F14" s="7">
-        <v>1</v>
-      </c>
-      <c r="G14" s="8">
+      <c r="F14" s="5">
+        <v>1</v>
+      </c>
+      <c r="G14" s="6">
         <f t="shared" si="0"/>
         <v>1400</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="H14" s="3" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="4">
+      <c r="A15" s="2">
         <v>13</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="4">
         <v>12</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="5">
         <v>50</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="6">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="H15" s="3" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" s="4">
+      <c r="A16" s="2">
         <v>14</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="4">
         <v>10</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F16" s="5">
         <v>30</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="6">
         <f t="shared" si="0"/>
         <v>300</v>
       </c>
-      <c r="H16" s="5" t="s">
+      <c r="H16" s="3" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" s="4">
+      <c r="A17" s="2">
         <v>15</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="4">
         <v>12</v>
       </c>
-      <c r="F17" s="7">
+      <c r="F17" s="5">
         <v>20</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="6">
         <f t="shared" si="0"/>
         <v>240</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H17" s="3" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" s="4">
+      <c r="A18" s="2">
         <v>16</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="4">
         <v>60</v>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="5">
         <v>2</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="6">
         <f t="shared" si="0"/>
         <v>120</v>
       </c>
-      <c r="H18" s="5" t="s">
+      <c r="H18" s="3" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="4">
+      <c r="A19" s="2">
         <v>17</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="4">
         <v>350</v>
       </c>
-      <c r="F19" s="7">
-        <v>1</v>
-      </c>
-      <c r="G19" s="8">
+      <c r="F19" s="5">
+        <v>1</v>
+      </c>
+      <c r="G19" s="6">
         <f t="shared" si="0"/>
         <v>350</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="H19" s="3" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="4">
+      <c r="A20" s="2">
         <v>18</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="4">
         <v>1200</v>
       </c>
-      <c r="F20" s="7">
-        <v>1</v>
-      </c>
-      <c r="G20" s="8">
+      <c r="F20" s="5">
+        <v>1</v>
+      </c>
+      <c r="G20" s="6">
         <f t="shared" si="0"/>
         <v>1200</v>
       </c>
-      <c r="H20" s="5" t="s">
+      <c r="H20" s="3" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="9"/>
-      <c r="B21" s="10" t="s">
+      <c r="A21" s="7"/>
+      <c r="B21" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="11">
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="9">
         <f>SUM(G3:G20)</f>
         <v>12870</v>
       </c>
-      <c r="H21" s="9"/>
+      <c r="H21" s="7"/>
     </row>
     <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" s="4">
-        <v>1</v>
-      </c>
-      <c r="B24" s="5" t="s">
+      <c r="A24" s="2">
+        <v>1</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E24" s="6">
+      <c r="E24" s="4">
         <v>850</v>
       </c>
-      <c r="F24" s="7">
-        <v>1</v>
-      </c>
-      <c r="G24" s="8">
+      <c r="F24" s="5">
+        <v>1</v>
+      </c>
+      <c r="G24" s="6">
         <f t="shared" ref="G24:G46" si="1">E24*F24</f>
         <v>850</v>
       </c>
-      <c r="H24" s="5" t="s">
+      <c r="H24" s="3" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="4">
+      <c r="A25" s="2">
         <v>2</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="D25" s="4" t="s">
+      <c r="B25" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="4">
         <v>1100</v>
       </c>
-      <c r="F25" s="7">
-        <v>1</v>
-      </c>
-      <c r="G25" s="8">
+      <c r="F25" s="5">
+        <v>1</v>
+      </c>
+      <c r="G25" s="6">
         <f t="shared" si="1"/>
         <v>1100</v>
       </c>
-      <c r="H25" s="5" t="s">
+      <c r="H25" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" s="2">
+        <v>3</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" s="4">
+      <c r="D26" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E26" s="4">
+        <v>35</v>
+      </c>
+      <c r="F26" s="5">
         <v>3</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E26" s="6">
-        <v>35</v>
-      </c>
-      <c r="F26" s="7">
-        <v>3</v>
-      </c>
-      <c r="G26" s="8">
+      <c r="G26" s="6">
         <f t="shared" si="1"/>
         <v>105</v>
       </c>
-      <c r="H26" s="5" t="s">
+      <c r="H26" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" s="2">
+        <v>4</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="4">
-        <v>4</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="4">
         <v>220</v>
       </c>
-      <c r="F27" s="7">
-        <v>1</v>
-      </c>
-      <c r="G27" s="8">
+      <c r="F27" s="5">
+        <v>1</v>
+      </c>
+      <c r="G27" s="6">
         <f t="shared" si="1"/>
         <v>220</v>
       </c>
-      <c r="H27" s="5" t="s">
+      <c r="H27" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" s="2">
+        <v>5</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A28" s="4">
-        <v>5</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E28" s="4">
         <v>600</v>
       </c>
-      <c r="F28" s="7">
-        <v>1</v>
-      </c>
-      <c r="G28" s="8">
+      <c r="F28" s="5">
+        <v>1</v>
+      </c>
+      <c r="G28" s="6">
         <f t="shared" si="1"/>
         <v>600</v>
       </c>
-      <c r="H28" s="5" t="s">
+      <c r="H28" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29" s="2">
+        <v>6</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" s="4">
-        <v>6</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="4">
         <v>45</v>
       </c>
-      <c r="F29" s="7">
-        <v>1</v>
-      </c>
-      <c r="G29" s="8">
+      <c r="F29" s="5">
+        <v>1</v>
+      </c>
+      <c r="G29" s="6">
         <f t="shared" si="1"/>
         <v>45</v>
       </c>
-      <c r="H29" s="5" t="s">
+      <c r="H29" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" s="2">
+        <v>7</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A30" s="4">
-        <v>7</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E30" s="6">
+      <c r="E30" s="4">
         <v>25</v>
       </c>
-      <c r="F30" s="7">
+      <c r="F30" s="5">
         <v>2</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G30" s="6">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="H30" s="5" t="s">
+      <c r="H30" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31" s="2">
+        <v>8</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A31" s="4">
-        <v>8</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="4">
         <v>40</v>
       </c>
-      <c r="F31" s="7">
-        <v>1</v>
-      </c>
-      <c r="G31" s="8">
+      <c r="F31" s="5">
+        <v>1</v>
+      </c>
+      <c r="G31" s="6">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="H31" s="5" t="s">
+      <c r="H31" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A32" s="2">
+        <v>9</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A32" s="4">
-        <v>9</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="D32" s="4" t="s">
+      <c r="D32" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E32" s="6">
+      <c r="E32" s="4">
         <v>35</v>
       </c>
-      <c r="F32" s="7">
-        <v>1</v>
-      </c>
-      <c r="G32" s="8">
+      <c r="F32" s="5">
+        <v>1</v>
+      </c>
+      <c r="G32" s="6">
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
-      <c r="H32" s="5" t="s">
+      <c r="H32" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A33" s="2">
+        <v>10</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A33" s="4">
-        <v>10</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="D33" s="4" t="s">
+      <c r="D33" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E33" s="6">
+      <c r="E33" s="4">
         <v>25</v>
       </c>
-      <c r="F33" s="7">
+      <c r="F33" s="5">
         <v>4</v>
       </c>
-      <c r="G33" s="8">
+      <c r="G33" s="6">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="H33" s="5" t="s">
+      <c r="H33" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A34" s="2">
+        <v>11</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A34" s="4">
-        <v>11</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E34" s="6">
+      <c r="E34" s="4">
         <v>20</v>
       </c>
-      <c r="F34" s="7">
+      <c r="F34" s="5">
         <v>2</v>
       </c>
-      <c r="G34" s="8">
+      <c r="G34" s="6">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="H34" s="5" t="s">
+      <c r="H34" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A35" s="2">
+        <v>12</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C35" s="3" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A35" s="4">
-        <v>12</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="D35" s="4" t="s">
+      <c r="D35" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E35" s="6">
+      <c r="E35" s="4">
         <v>90</v>
       </c>
-      <c r="F35" s="7">
-        <v>1</v>
-      </c>
-      <c r="G35" s="8">
+      <c r="F35" s="5">
+        <v>1</v>
+      </c>
+      <c r="G35" s="6">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="H35" s="5" t="s">
+      <c r="H35" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A36" s="2">
+        <v>13</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C36" s="3" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A36" s="4">
-        <v>13</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D36" s="4" t="s">
+      <c r="D36" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E36" s="6">
+      <c r="E36" s="4">
         <v>25</v>
       </c>
-      <c r="F36" s="7">
+      <c r="F36" s="5">
         <v>2</v>
       </c>
-      <c r="G36" s="8">
+      <c r="G36" s="6">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="H36" s="5" t="s">
+      <c r="H36" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A37" s="2">
+        <v>14</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C37" s="3" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37" s="4">
-        <v>14</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="D37" s="4" t="s">
+      <c r="D37" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E37" s="6">
+      <c r="E37" s="4">
         <v>1200</v>
       </c>
-      <c r="F37" s="7">
-        <v>1</v>
-      </c>
-      <c r="G37" s="8">
+      <c r="F37" s="5">
+        <v>1</v>
+      </c>
+      <c r="G37" s="6">
         <f t="shared" si="1"/>
         <v>1200</v>
       </c>
-      <c r="H37" s="5" t="s">
+      <c r="H37" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A38" s="2">
+        <v>15</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A38" s="4">
-        <v>15</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="D38" s="4" t="s">
+      <c r="D38" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E38" s="6">
+      <c r="E38" s="4">
         <v>50</v>
       </c>
-      <c r="F38" s="7">
-        <v>1</v>
-      </c>
-      <c r="G38" s="8">
+      <c r="F38" s="5">
+        <v>1</v>
+      </c>
+      <c r="G38" s="6">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="H38" s="5" t="s">
+      <c r="H38" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A39" s="2">
+        <v>16</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A39" s="4">
-        <v>16</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="D39" s="4" t="s">
+      <c r="D39" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E39" s="6">
+      <c r="E39" s="4">
         <v>320</v>
       </c>
-      <c r="F39" s="7">
-        <v>1</v>
-      </c>
-      <c r="G39" s="8">
+      <c r="F39" s="5">
+        <v>1</v>
+      </c>
+      <c r="G39" s="6">
         <f t="shared" si="1"/>
         <v>320</v>
       </c>
-      <c r="H39" s="5" t="s">
+      <c r="H39" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A40" s="2">
+        <v>17</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A40" s="4">
-        <v>17</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="D40" s="4" t="s">
+      <c r="D40" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E40" s="6">
+      <c r="E40" s="4">
         <v>8</v>
       </c>
-      <c r="F40" s="7">
+      <c r="F40" s="5">
         <v>6</v>
       </c>
-      <c r="G40" s="8">
+      <c r="G40" s="6">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="H40" s="5" t="s">
+      <c r="H40" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A41" s="2">
+        <v>18</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C41" s="3" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A41" s="4">
-        <v>18</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="D41" s="4" t="s">
+      <c r="D41" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E41" s="6">
+      <c r="E41" s="4">
         <v>5</v>
       </c>
-      <c r="F41" s="7">
+      <c r="F41" s="5">
         <v>10</v>
       </c>
-      <c r="G41" s="8">
+      <c r="G41" s="6">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="H41" s="5" t="s">
+      <c r="H41" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A42" s="2">
+        <v>19</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C42" s="3" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A42" s="4">
-        <v>19</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="D42" s="4" t="s">
+      <c r="D42" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E42" s="6">
+      <c r="E42" s="4">
         <v>250</v>
       </c>
-      <c r="F42" s="7">
-        <v>1</v>
-      </c>
-      <c r="G42" s="8">
+      <c r="F42" s="5">
+        <v>1</v>
+      </c>
+      <c r="G42" s="6">
         <f t="shared" si="1"/>
         <v>250</v>
       </c>
-      <c r="H42" s="5" t="s">
+      <c r="H42" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A43" s="2">
+        <v>20</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A43" s="4">
-        <v>20</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="D43" s="4" t="s">
+      <c r="D43" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E43" s="6">
+      <c r="E43" s="4">
         <v>280</v>
       </c>
-      <c r="F43" s="7">
-        <v>1</v>
-      </c>
-      <c r="G43" s="8">
+      <c r="F43" s="5">
+        <v>1</v>
+      </c>
+      <c r="G43" s="6">
         <f t="shared" si="1"/>
         <v>280</v>
       </c>
-      <c r="H43" s="5" t="s">
+      <c r="H43" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A44" s="2">
+        <v>21</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C44" s="3" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A44" s="4">
-        <v>21</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D44" s="4" t="s">
+      <c r="D44" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E44" s="6">
+      <c r="E44" s="4">
         <v>6</v>
       </c>
-      <c r="F44" s="7">
+      <c r="F44" s="5">
         <v>12</v>
       </c>
-      <c r="G44" s="8">
+      <c r="G44" s="6">
         <f t="shared" si="1"/>
         <v>72</v>
       </c>
-      <c r="H44" s="5" t="s">
+      <c r="H44" s="3" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A45" s="2">
+        <v>22</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C45" s="3" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A45" s="4">
-        <v>22</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="D45" s="4" t="s">
+      <c r="D45" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E45" s="6">
+      <c r="E45" s="4">
         <v>30</v>
       </c>
-      <c r="F45" s="7">
+      <c r="F45" s="5">
         <v>4</v>
       </c>
-      <c r="G45" s="8">
+      <c r="G45" s="6">
         <f t="shared" si="1"/>
         <v>120</v>
       </c>
-      <c r="H45" s="5" t="s">
+      <c r="H45" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="25" x14ac:dyDescent="0.35">
+      <c r="A46" s="2">
+        <v>23</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C46" s="3" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A46" s="4">
-        <v>23</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D46" s="4" t="s">
+      <c r="D46" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E46" s="6">
+      <c r="E46" s="4">
         <v>280</v>
       </c>
-      <c r="F46" s="7">
-        <v>1</v>
-      </c>
-      <c r="G46" s="8">
+      <c r="F46" s="5">
+        <v>1</v>
+      </c>
+      <c r="G46" s="6">
         <f t="shared" si="1"/>
         <v>280</v>
       </c>
-      <c r="H46" s="5" t="s">
-        <v>139</v>
+      <c r="H46" s="3" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A47" s="9"/>
-      <c r="B47" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="C47" s="9"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="9"/>
-      <c r="G47" s="11">
+      <c r="A47" s="7"/>
+      <c r="B47" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C47" s="7"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="9">
         <f>SUM(G24:G46)</f>
         <v>5995</v>
       </c>
-      <c r="H47" s="9"/>
+      <c r="H47" s="7"/>
     </row>
     <row r="49" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="2" t="s">
+      <c r="A49" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="B49" s="14"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="14"/>
+      <c r="F49" s="14"/>
+      <c r="G49" s="14"/>
+      <c r="H49" s="14"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A50" s="2">
+        <v>1</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C50" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-      <c r="G49" s="2"/>
-      <c r="H49" s="2"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A50" s="4">
-        <v>1</v>
-      </c>
-      <c r="B50" s="5" t="s">
+      <c r="D50" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C50" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="E50" s="6">
+      <c r="E50" s="4">
         <v>1900</v>
       </c>
-      <c r="F50" s="7">
-        <v>1</v>
-      </c>
-      <c r="G50" s="8">
+      <c r="F50" s="5">
+        <v>1</v>
+      </c>
+      <c r="G50" s="6">
         <f t="shared" ref="G50:G55" si="2">E50*F50</f>
         <v>1900</v>
       </c>
-      <c r="H50" s="5" t="s">
+      <c r="H50" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A51" s="2">
+        <v>2</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A51" s="4">
-        <v>2</v>
-      </c>
-      <c r="B51" s="5" t="s">
+      <c r="D51" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="C51" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="E51" s="6">
+      <c r="E51" s="4">
         <v>700</v>
       </c>
-      <c r="F51" s="7">
-        <v>1</v>
-      </c>
-      <c r="G51" s="8">
+      <c r="F51" s="5">
+        <v>1</v>
+      </c>
+      <c r="G51" s="6">
         <f t="shared" si="2"/>
         <v>700</v>
       </c>
-      <c r="H51" s="5" t="s">
+      <c r="H51" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A52" s="2">
+        <v>3</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C52" s="3" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" s="4">
-        <v>3</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="D52" s="4" t="s">
+      <c r="D52" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E52" s="6">
+      <c r="E52" s="4">
         <v>600</v>
       </c>
-      <c r="F52" s="7">
-        <v>1</v>
-      </c>
-      <c r="G52" s="8">
+      <c r="F52" s="5">
+        <v>1</v>
+      </c>
+      <c r="G52" s="6">
         <f t="shared" si="2"/>
         <v>600</v>
       </c>
-      <c r="H52" s="5" t="s">
+      <c r="H52" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A53" s="2">
+        <v>4</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C53" s="3" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A53" s="4">
-        <v>4</v>
-      </c>
-      <c r="B53" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="D53" s="4" t="s">
+      <c r="D53" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E53" s="6">
+      <c r="E53" s="4">
         <v>350</v>
       </c>
-      <c r="F53" s="7">
-        <v>1</v>
-      </c>
-      <c r="G53" s="8">
+      <c r="F53" s="5">
+        <v>1</v>
+      </c>
+      <c r="G53" s="6">
         <f t="shared" si="2"/>
         <v>350</v>
       </c>
-      <c r="H53" s="5" t="s">
+      <c r="H53" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A54" s="2">
+        <v>5</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C54" s="3" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A54" s="4">
-        <v>5</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="D54" s="4" t="s">
+      <c r="D54" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E54" s="6">
+      <c r="E54" s="4">
         <v>280</v>
       </c>
-      <c r="F54" s="7">
-        <v>1</v>
-      </c>
-      <c r="G54" s="8">
+      <c r="F54" s="5">
+        <v>1</v>
+      </c>
+      <c r="G54" s="6">
         <f t="shared" si="2"/>
         <v>280</v>
       </c>
-      <c r="H54" s="5" t="s">
+      <c r="H54" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A55" s="2">
+        <v>6</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C55" s="3" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A55" s="4">
-        <v>6</v>
-      </c>
-      <c r="B55" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="C55" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="D55" s="4" t="s">
+      <c r="D55" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E55" s="6">
+      <c r="E55" s="4">
         <v>280</v>
       </c>
-      <c r="F55" s="7">
-        <v>1</v>
-      </c>
-      <c r="G55" s="8">
+      <c r="F55" s="5">
+        <v>1</v>
+      </c>
+      <c r="G55" s="6">
         <f t="shared" si="2"/>
         <v>280</v>
       </c>
-      <c r="H55" s="5" t="s">
-        <v>161</v>
+      <c r="H55" s="3" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A56" s="9"/>
-      <c r="B56" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="C56" s="9"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="9"/>
-      <c r="F56" s="9"/>
-      <c r="G56" s="11">
+      <c r="A56" s="7"/>
+      <c r="B56" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="C56" s="7"/>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="9">
         <f>SUM(G50:G55)</f>
         <v>4110</v>
       </c>
-      <c r="H56" s="9"/>
+      <c r="H56" s="7"/>
     </row>
     <row r="58" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="2" t="s">
+      <c r="A58" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="B58" s="14"/>
+      <c r="C58" s="14"/>
+      <c r="D58" s="14"/>
+      <c r="E58" s="14"/>
+      <c r="F58" s="14"/>
+      <c r="G58" s="14"/>
+      <c r="H58" s="14"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A59" s="2">
+        <v>1</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C59" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
-      <c r="F58" s="2"/>
-      <c r="G58" s="2"/>
-      <c r="H58" s="2"/>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A59" s="4">
-        <v>1</v>
-      </c>
-      <c r="B59" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="D59" s="4" t="s">
+      <c r="D59" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E59" s="6">
+      <c r="E59" s="4">
         <v>250</v>
       </c>
-      <c r="F59" s="7">
-        <v>1</v>
-      </c>
-      <c r="G59" s="8">
+      <c r="F59" s="5">
+        <v>1</v>
+      </c>
+      <c r="G59" s="6">
         <f t="shared" ref="G59:G65" si="3">E59*F59</f>
         <v>250</v>
       </c>
-      <c r="H59" s="5" t="s">
+      <c r="H59" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A60" s="2">
+        <v>2</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C60" s="3" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A60" s="4">
-        <v>2</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="D60" s="4" t="s">
+      <c r="D60" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E60" s="6">
+      <c r="E60" s="4">
         <v>350</v>
       </c>
-      <c r="F60" s="7">
-        <v>1</v>
-      </c>
-      <c r="G60" s="8">
+      <c r="F60" s="5">
+        <v>1</v>
+      </c>
+      <c r="G60" s="6">
         <f t="shared" si="3"/>
         <v>350</v>
       </c>
-      <c r="H60" s="5" t="s">
+      <c r="H60" s="3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A61" s="2">
+        <v>3</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C61" s="3" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A61" s="4">
-        <v>3</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="D61" s="4" t="s">
+      <c r="D61" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E61" s="6">
+      <c r="E61" s="4">
         <v>250</v>
       </c>
-      <c r="F61" s="7">
-        <v>1</v>
-      </c>
-      <c r="G61" s="8">
+      <c r="F61" s="5">
+        <v>1</v>
+      </c>
+      <c r="G61" s="6">
         <f t="shared" si="3"/>
         <v>250</v>
       </c>
-      <c r="H61" s="5" t="s">
+      <c r="H61" s="3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A62" s="2">
+        <v>4</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C62" s="3" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A62" s="4">
-        <v>4</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="C62" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="D62" s="4" t="s">
+      <c r="D62" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E62" s="6">
+      <c r="E62" s="4">
         <v>120</v>
       </c>
-      <c r="F62" s="7">
-        <v>1</v>
-      </c>
-      <c r="G62" s="8">
+      <c r="F62" s="5">
+        <v>1</v>
+      </c>
+      <c r="G62" s="6">
         <f t="shared" si="3"/>
         <v>120</v>
       </c>
-      <c r="H62" s="5" t="s">
+      <c r="H62" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A63" s="2">
+        <v>5</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C63" s="3" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A63" s="4">
-        <v>5</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="D63" s="4" t="s">
+      <c r="D63" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E63" s="6">
+      <c r="E63" s="4">
         <v>180</v>
       </c>
-      <c r="F63" s="7">
-        <v>1</v>
-      </c>
-      <c r="G63" s="8">
+      <c r="F63" s="5">
+        <v>1</v>
+      </c>
+      <c r="G63" s="6">
         <f t="shared" si="3"/>
         <v>180</v>
       </c>
-      <c r="H63" s="5" t="s">
+      <c r="H63" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A64" s="2">
+        <v>6</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="C64" s="3" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A64" s="4">
-        <v>6</v>
-      </c>
-      <c r="B64" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="C64" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D64" s="4" t="s">
+      <c r="D64" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E64" s="6">
+      <c r="E64" s="4">
         <v>450</v>
       </c>
-      <c r="F64" s="7">
-        <v>1</v>
-      </c>
-      <c r="G64" s="8">
+      <c r="F64" s="5">
+        <v>1</v>
+      </c>
+      <c r="G64" s="6">
         <f t="shared" si="3"/>
         <v>450</v>
       </c>
-      <c r="H64" s="5" t="s">
+      <c r="H64" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A65" s="2">
+        <v>7</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="C65" s="3" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A65" s="4">
-        <v>7</v>
-      </c>
-      <c r="B65" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="C65" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="D65" s="4" t="s">
+      <c r="D65" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E65" s="6">
+      <c r="E65" s="4">
         <v>250</v>
       </c>
-      <c r="F65" s="7">
-        <v>1</v>
-      </c>
-      <c r="G65" s="8">
+      <c r="F65" s="5">
+        <v>1</v>
+      </c>
+      <c r="G65" s="6">
         <f t="shared" si="3"/>
         <v>250</v>
       </c>
-      <c r="H65" s="5" t="s">
-        <v>184</v>
+      <c r="H65" s="3" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A66" s="9"/>
-      <c r="B66" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="9"/>
-      <c r="F66" s="9"/>
-      <c r="G66" s="11">
+      <c r="A66" s="7"/>
+      <c r="B66" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C66" s="7"/>
+      <c r="D66" s="7"/>
+      <c r="E66" s="7"/>
+      <c r="F66" s="7"/>
+      <c r="G66" s="9">
         <f>SUM(G59:G65)</f>
         <v>1850</v>
       </c>
-      <c r="H66" s="9"/>
+      <c r="H66" s="7"/>
     </row>
     <row r="68" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A68" s="9"/>
-      <c r="B68" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="C68" s="9"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="9"/>
-      <c r="F68" s="9"/>
-      <c r="G68" s="13">
+      <c r="A68" s="7"/>
+      <c r="B68" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="C68" s="7"/>
+      <c r="D68" s="7"/>
+      <c r="E68" s="7"/>
+      <c r="F68" s="7"/>
+      <c r="G68" s="11">
         <f>G21+G47+G56+G66</f>
         <v>24825</v>
       </c>
-      <c r="H68" s="9"/>
+      <c r="H68" s="7"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B70" s="14" t="s">
+      <c r="B70" s="12" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B71" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="C71" s="13"/>
+      <c r="D71" s="13"/>
+      <c r="E71" s="13"/>
+      <c r="F71" s="13"/>
+      <c r="G71" s="13"/>
+      <c r="H71" s="13"/>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B72" s="13" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B71" s="1" t="s">
+      <c r="C72" s="13"/>
+      <c r="D72" s="13"/>
+      <c r="E72" s="13"/>
+      <c r="F72" s="13"/>
+      <c r="G72" s="13"/>
+      <c r="H72" s="13"/>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B73" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="C71" s="1"/>
-      <c r="D71" s="1"/>
-      <c r="E71" s="1"/>
-      <c r="F71" s="1"/>
-      <c r="G71" s="1"/>
-      <c r="H71" s="1"/>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B72" s="1" t="s">
+      <c r="C73" s="13"/>
+      <c r="D73" s="13"/>
+      <c r="E73" s="13"/>
+      <c r="F73" s="13"/>
+      <c r="G73" s="13"/>
+      <c r="H73" s="13"/>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B74" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="C72" s="1"/>
-      <c r="D72" s="1"/>
-      <c r="E72" s="1"/>
-      <c r="F72" s="1"/>
-      <c r="G72" s="1"/>
-      <c r="H72" s="1"/>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B73" s="1" t="s">
+      <c r="C74" s="13"/>
+      <c r="D74" s="13"/>
+      <c r="E74" s="13"/>
+      <c r="F74" s="13"/>
+      <c r="G74" s="13"/>
+      <c r="H74" s="13"/>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B75" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="C73" s="1"/>
-      <c r="D73" s="1"/>
-      <c r="E73" s="1"/>
-      <c r="F73" s="1"/>
-      <c r="G73" s="1"/>
-      <c r="H73" s="1"/>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B74" s="1" t="s">
+      <c r="C75" s="13"/>
+      <c r="D75" s="13"/>
+      <c r="E75" s="13"/>
+      <c r="F75" s="13"/>
+      <c r="G75" s="13"/>
+      <c r="H75" s="13"/>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B76" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="C74" s="1"/>
-      <c r="D74" s="1"/>
-      <c r="E74" s="1"/>
-      <c r="F74" s="1"/>
-      <c r="G74" s="1"/>
-      <c r="H74" s="1"/>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B75" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="C75" s="1"/>
-      <c r="D75" s="1"/>
-      <c r="E75" s="1"/>
-      <c r="F75" s="1"/>
-      <c r="G75" s="1"/>
-      <c r="H75" s="1"/>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B76" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="C76" s="1"/>
-      <c r="D76" s="1"/>
-      <c r="E76" s="1"/>
-      <c r="F76" s="1"/>
-      <c r="G76" s="1"/>
-      <c r="H76" s="1"/>
+      <c r="C76" s="13"/>
+      <c r="D76" s="13"/>
+      <c r="E76" s="13"/>
+      <c r="F76" s="13"/>
+      <c r="G76" s="13"/>
+      <c r="H76" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A58:H58"/>
+    <mergeCell ref="B71:H71"/>
     <mergeCell ref="B72:H72"/>
     <mergeCell ref="B73:H73"/>
     <mergeCell ref="B74:H74"/>
     <mergeCell ref="B75:H75"/>
     <mergeCell ref="B76:H76"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A49:H49"/>
-    <mergeCell ref="A58:H58"/>
-    <mergeCell ref="B71:H71"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>